<commit_message>
Add scheduled reports and Rocket75 import workflow
</commit_message>
<xml_diff>
--- a/HRMI-processing-times.xlsx
+++ b/HRMI-processing-times.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="เวลาประมวลผล" sheetId="1" r:id="R135a5302b0b44032"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="เวลาประมวลผล" sheetId="1" r:id="Re4c7d3d2c0d44dc3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,10 +13,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
-    <x:numFmt numFmtId="200" formatCode="dd/mm/yyyy"/>
-    <x:numFmt numFmtId="201" formatCode="dd/mm/yyyy hh:mm:ss"/>
-    <x:numFmt numFmtId="202" formatCode="[h]:mm:ss"/>
+  <x:numFmts count="2">
+    <x:numFmt numFmtId="200" formatCode="dd/mm/yyyy hh:mm:ss"/>
+    <x:numFmt numFmtId="201" formatCode="[h]:mm:ss"/>
   </x:numFmts>
   <x:fonts count="6">
     <x:font>
@@ -135,7 +134,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="38">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -175,9 +174,6 @@
     <x:xf numFmtId="201" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="202" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -187,9 +183,6 @@
     <x:xf numFmtId="201" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="202" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -199,9 +192,6 @@
     <x:xf numFmtId="201" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="202" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -211,9 +201,6 @@
     <x:xf numFmtId="201" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="202" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -221,9 +208,6 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="4" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="4" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -461,7 +445,7 @@
   <x:cols>
     <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="23" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="23" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
@@ -470,14 +454,14 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="36"/>
-      <x:c r="B1" s="36"/>
-      <x:c r="C1" s="36"/>
-      <x:c r="D1" s="36"/>
-      <x:c r="E1" s="36"/>
-      <x:c r="F1" s="36"/>
-      <x:c r="G1" s="36"/>
-      <x:c r="H1" s="37"/>
+      <x:c r="A1" s="31"/>
+      <x:c r="B1" s="31"/>
+      <x:c r="C1" s="31"/>
+      <x:c r="D1" s="31"/>
+      <x:c r="E1" s="31"/>
+      <x:c r="F1" s="31"/>
+      <x:c r="G1" s="31"/>
+      <x:c r="H1" s="32"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2" t="str">
@@ -502,7 +486,7 @@
         <x:v>สาขา</x:v>
       </x:c>
       <x:c r="C4" s="13" t="str">
-        <x:v>วันที่ประมวลผล</x:v>
+        <x:v>ช่วงวันที่ประมวลผล</x:v>
       </x:c>
       <x:c r="D4" s="13" t="str">
         <x:v>เวลาเริ่ม</x:v>
@@ -527,16 +511,16 @@
       <x:c r="B5" s="16" t="str">
         <x:v>[BB]</x:v>
       </x:c>
-      <x:c r="C5" s="17" t="d">
-        <x:v>2026-10-08T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D5" s="18" t="d">
+      <x:c r="C5" s="16" t="str">
+        <x:v>08/10/2026</x:v>
+      </x:c>
+      <x:c r="D5" s="17" t="d">
         <x:v>2026-10-10T09:41:22.874Z</x:v>
       </x:c>
-      <x:c r="E5" s="18" t="d">
+      <x:c r="E5" s="17" t="d">
         <x:v>2026-10-10T09:48:40.904Z</x:v>
       </x:c>
-      <x:c r="F5" s="19" t="n">
+      <x:c r="F5" s="18" t="n">
         <x:v>0.005069791666666666</x:v>
       </x:c>
       <x:c r="G5" s="16" t="str">
@@ -547,28 +531,28 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="20" t="str">
+      <x:c r="A6" s="19" t="str">
         <x:v>20261010-094118-026012</x:v>
       </x:c>
-      <x:c r="B6" s="20" t="str">
+      <x:c r="B6" s="19" t="str">
         <x:v>[BK]</x:v>
       </x:c>
-      <x:c r="C6" s="21" t="d">
-        <x:v>2026-10-08T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D6" s="22" t="d">
+      <x:c r="C6" s="19" t="str">
+        <x:v>08/10/2026</x:v>
+      </x:c>
+      <x:c r="D6" s="20" t="d">
         <x:v>2026-10-10T09:48:46.590Z</x:v>
       </x:c>
-      <x:c r="E6" s="22" t="d">
+      <x:c r="E6" s="20" t="d">
         <x:v>2026-10-10T10:00:11.179Z</x:v>
       </x:c>
-      <x:c r="F6" s="23" t="n">
+      <x:c r="F6" s="21" t="n">
         <x:v>0.00792349537037037</x:v>
       </x:c>
-      <x:c r="G6" s="20" t="str">
-        <x:v>สำเร็จ</x:v>
-      </x:c>
-      <x:c r="H6" s="20" t="str">
+      <x:c r="G6" s="19" t="str">
+        <x:v>สำเร็จ</x:v>
+      </x:c>
+      <x:c r="H6" s="19" t="str">
         <x:v>เสร็จตามขั้นตอนที่กำหนด</x:v>
       </x:c>
     </x:row>
@@ -579,16 +563,16 @@
       <x:c r="B7" s="16" t="str">
         <x:v>[NTS]</x:v>
       </x:c>
-      <x:c r="C7" s="17" t="d">
-        <x:v>2026-10-08T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D7" s="18" t="d">
+      <x:c r="C7" s="16" t="str">
+        <x:v>08/10/2026</x:v>
+      </x:c>
+      <x:c r="D7" s="17" t="d">
         <x:v>2026-10-10T10:00:18.549Z</x:v>
       </x:c>
-      <x:c r="E7" s="18" t="d">
+      <x:c r="E7" s="17" t="d">
         <x:v>2026-10-10T10:01:22.419Z</x:v>
       </x:c>
-      <x:c r="F7" s="19" t="n">
+      <x:c r="F7" s="18" t="n">
         <x:v>0.0007392361111111111</x:v>
       </x:c>
       <x:c r="G7" s="16" t="str">
@@ -599,28 +583,28 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="20" t="str">
+      <x:c r="A8" s="19" t="str">
         <x:v>20261010-094118-026012</x:v>
       </x:c>
-      <x:c r="B8" s="20" t="str">
+      <x:c r="B8" s="19" t="str">
         <x:v>[PK]</x:v>
       </x:c>
-      <x:c r="C8" s="21" t="d">
-        <x:v>2026-10-08T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D8" s="22" t="d">
+      <x:c r="C8" s="19" t="str">
+        <x:v>08/10/2026</x:v>
+      </x:c>
+      <x:c r="D8" s="20" t="d">
         <x:v>2026-10-10T10:01:28.773Z</x:v>
       </x:c>
-      <x:c r="E8" s="22" t="d">
+      <x:c r="E8" s="20" t="d">
         <x:v>2026-10-10T10:03:59.193Z</x:v>
       </x:c>
-      <x:c r="F8" s="23" t="n">
+      <x:c r="F8" s="21" t="n">
         <x:v>0.001740972222222222</x:v>
       </x:c>
-      <x:c r="G8" s="20" t="str">
-        <x:v>สำเร็จ</x:v>
-      </x:c>
-      <x:c r="H8" s="20" t="str">
+      <x:c r="G8" s="19" t="str">
+        <x:v>สำเร็จ</x:v>
+      </x:c>
+      <x:c r="H8" s="19" t="str">
         <x:v>เสร็จตามขั้นตอนที่กำหนด</x:v>
       </x:c>
     </x:row>
@@ -631,16 +615,16 @@
       <x:c r="B9" s="16" t="str">
         <x:v>[SM]</x:v>
       </x:c>
-      <x:c r="C9" s="17" t="d">
-        <x:v>2026-10-08T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D9" s="18" t="d">
+      <x:c r="C9" s="16" t="str">
+        <x:v>08/10/2026</x:v>
+      </x:c>
+      <x:c r="D9" s="17" t="d">
         <x:v>2026-10-10T10:04:05.491Z</x:v>
       </x:c>
-      <x:c r="E9" s="18" t="d">
+      <x:c r="E9" s="17" t="d">
         <x:v>2026-10-10T10:06:16.093Z</x:v>
       </x:c>
-      <x:c r="F9" s="19" t="n">
+      <x:c r="F9" s="18" t="n">
         <x:v>0.0015115972222222223</x:v>
       </x:c>
       <x:c r="G9" s="16" t="str">
@@ -651,28 +635,548 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="32" t="str">
+      <x:c r="A10" s="28" t="str">
         <x:v>20261010-094118-026012</x:v>
       </x:c>
-      <x:c r="B10" s="32" t="str">
+      <x:c r="B10" s="28" t="str">
         <x:v>สรุปรอบ</x:v>
       </x:c>
-      <x:c r="C10" s="33" t="d">
-        <x:v>2026-10-08T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D10" s="34" t="d">
+      <x:c r="C10" s="28" t="str">
+        <x:v>08/10/2026</x:v>
+      </x:c>
+      <x:c r="D10" s="29" t="d">
         <x:v>2026-10-10T09:41:22.874Z</x:v>
       </x:c>
-      <x:c r="E10" s="34" t="d">
+      <x:c r="E10" s="29" t="d">
         <x:v>2026-10-10T10:06:16.093Z</x:v>
       </x:c>
-      <x:c r="F10" s="35" t="n">
+      <x:c r="F10" s="30" t="n">
         <x:v>0.017282627314814815</x:v>
       </x:c>
-      <x:c r="G10" s="32" t="str">
+      <x:c r="G10" s="28" t="str">
         <x:v>สำเร็จครบ 5 สาขา</x:v>
       </x:c>
-      <x:c r="H10" s="32" t="str">
+      <x:c r="H10" s="28" t="str">
+        <x:v>รวมตั้งแต่เริ่ม [BB] ถึง Finish [SM]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="16" t="str">
+        <x:v>20261012-094707</x:v>
+      </x:c>
+      <x:c r="B11" s="16" t="str">
+        <x:v>[BB]</x:v>
+      </x:c>
+      <x:c r="C11" s="16" t="str">
+        <x:v>10/10/2026</x:v>
+      </x:c>
+      <x:c r="D11" s="17" t="d">
+        <x:v>2026-10-12T09:47:13.779Z</x:v>
+      </x:c>
+      <x:c r="E11" s="17" t="d">
+        <x:v>2026-10-12T09:47:25.009Z</x:v>
+      </x:c>
+      <x:c r="F11" s="18" t="n">
+        <x:v>0.00012997685185185185</x:v>
+      </x:c>
+      <x:c r="G11" s="16" t="str">
+        <x:v>ผิดพลาด</x:v>
+      </x:c>
+      <x:c r="H11" s="16" t="str">
+        <x:v>Handle 68352 is not a vaild window handle</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="19" t="str">
+        <x:v>20261012-104337</x:v>
+      </x:c>
+      <x:c r="B12" s="19" t="str">
+        <x:v>[BB]</x:v>
+      </x:c>
+      <x:c r="C12" s="19" t="str">
+        <x:v>09/10/2026 - 10/10/2026</x:v>
+      </x:c>
+      <x:c r="D12" s="20" t="d">
+        <x:v>2026-10-12T10:43:44.061Z</x:v>
+      </x:c>
+      <x:c r="E12" s="20" t="d">
+        <x:v>2026-10-12T10:51:20.996Z</x:v>
+      </x:c>
+      <x:c r="F12" s="21" t="n">
+        <x:v>0.005288599537037037</x:v>
+      </x:c>
+      <x:c r="G12" s="19" t="str">
+        <x:v>สำเร็จ</x:v>
+      </x:c>
+      <x:c r="H12" s="19" t="str">
+        <x:v>ประมวลผลและกด Finish แล้ว</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="16" t="str">
+        <x:v>20261012-104337</x:v>
+      </x:c>
+      <x:c r="B13" s="16" t="str">
+        <x:v>[BK]</x:v>
+      </x:c>
+      <x:c r="C13" s="16" t="str">
+        <x:v>09/10/2026 - 10/10/2026</x:v>
+      </x:c>
+      <x:c r="D13" s="17" t="d">
+        <x:v>2026-10-12T10:51:28.432Z</x:v>
+      </x:c>
+      <x:c r="E13" s="17" t="d">
+        <x:v>2026-10-12T11:04:00.629Z</x:v>
+      </x:c>
+      <x:c r="F13" s="18" t="n">
+        <x:v>0.008705995370370371</x:v>
+      </x:c>
+      <x:c r="G13" s="16" t="str">
+        <x:v>สำเร็จ</x:v>
+      </x:c>
+      <x:c r="H13" s="16" t="str">
+        <x:v>ประมวลผลและกด Finish แล้ว</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="19" t="str">
+        <x:v>20261012-104337</x:v>
+      </x:c>
+      <x:c r="B14" s="19" t="str">
+        <x:v>[NTS]</x:v>
+      </x:c>
+      <x:c r="C14" s="19" t="str">
+        <x:v>09/10/2026 - 10/10/2026</x:v>
+      </x:c>
+      <x:c r="D14" s="20" t="d">
+        <x:v>2026-10-12T11:04:08.299Z</x:v>
+      </x:c>
+      <x:c r="E14" s="20" t="d">
+        <x:v>2026-10-12T11:05:12.625Z</x:v>
+      </x:c>
+      <x:c r="F14" s="21" t="n">
+        <x:v>0.0007445138888888889</x:v>
+      </x:c>
+      <x:c r="G14" s="19" t="str">
+        <x:v>สำเร็จ</x:v>
+      </x:c>
+      <x:c r="H14" s="19" t="str">
+        <x:v>ประมวลผลและกด Finish แล้ว</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="16" t="str">
+        <x:v>20261012-104337</x:v>
+      </x:c>
+      <x:c r="B15" s="16" t="str">
+        <x:v>[PK]</x:v>
+      </x:c>
+      <x:c r="C15" s="16" t="str">
+        <x:v>09/10/2026 - 10/10/2026</x:v>
+      </x:c>
+      <x:c r="D15" s="17" t="d">
+        <x:v>2026-10-12T11:05:20.386Z</x:v>
+      </x:c>
+      <x:c r="E15" s="17" t="d">
+        <x:v>2026-10-12T11:07:40.503Z</x:v>
+      </x:c>
+      <x:c r="F15" s="18" t="n">
+        <x:v>0.001621724537037037</x:v>
+      </x:c>
+      <x:c r="G15" s="16" t="str">
+        <x:v>สำเร็จ</x:v>
+      </x:c>
+      <x:c r="H15" s="16" t="str">
+        <x:v>ประมวลผลและกด Finish แล้ว</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="19" t="str">
+        <x:v>20261012-104337</x:v>
+      </x:c>
+      <x:c r="B16" s="19" t="str">
+        <x:v>[SM]</x:v>
+      </x:c>
+      <x:c r="C16" s="19" t="str">
+        <x:v>09/10/2026 - 10/10/2026</x:v>
+      </x:c>
+      <x:c r="D16" s="20" t="d">
+        <x:v>2026-10-12T11:07:47.662Z</x:v>
+      </x:c>
+      <x:c r="E16" s="20" t="d">
+        <x:v>2026-10-12T11:10:02.335Z</x:v>
+      </x:c>
+      <x:c r="F16" s="21" t="n">
+        <x:v>0.0015587152777777778</x:v>
+      </x:c>
+      <x:c r="G16" s="19" t="str">
+        <x:v>สำเร็จ</x:v>
+      </x:c>
+      <x:c r="H16" s="19" t="str">
+        <x:v>ประมวลผลและกด Finish แล้ว</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="28" t="str">
+        <x:v>20261012-104337</x:v>
+      </x:c>
+      <x:c r="B17" s="28" t="str">
+        <x:v>สรุปรอบ</x:v>
+      </x:c>
+      <x:c r="C17" s="28" t="str">
+        <x:v>09/10/2026 - 10/10/2026</x:v>
+      </x:c>
+      <x:c r="D17" s="29" t="d">
+        <x:v>2026-10-12T10:43:44.061Z</x:v>
+      </x:c>
+      <x:c r="E17" s="29" t="d">
+        <x:v>2026-10-12T11:10:02.335Z</x:v>
+      </x:c>
+      <x:c r="F17" s="30" t="n">
+        <x:v>0.018267060185185185</x:v>
+      </x:c>
+      <x:c r="G17" s="28" t="str">
+        <x:v>สำเร็จครบ 5 สาขา</x:v>
+      </x:c>
+      <x:c r="H17" s="28" t="str">
+        <x:v>รวมตั้งแต่เริ่ม [BB] ถึง Finish [SM]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="19" t="str">
+        <x:v>20261012-161702</x:v>
+      </x:c>
+      <x:c r="B18" s="19" t="str">
+        <x:v>[BB]</x:v>
+      </x:c>
+      <x:c r="C18" s="19" t="str">
+        <x:v>10/10/2026</x:v>
+      </x:c>
+      <x:c r="D18" s="20" t="d">
+        <x:v>2026-10-12T16:17:06.526Z</x:v>
+      </x:c>
+      <x:c r="E18" s="20" t="d">
+        <x:v>2026-10-12T16:18:18.290Z</x:v>
+      </x:c>
+      <x:c r="F18" s="21" t="n">
+        <x:v>0.0008306134259259259</x:v>
+      </x:c>
+      <x:c r="G18" s="19" t="str">
+        <x:v>ผิดพลาด</x:v>
+      </x:c>
+      <x:c r="H18" s="19" t="str">
+        <x:v>ไม่พบหน้าต่างประมวลผลเวลา</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="16" t="str">
+        <x:v>20261013-090231</x:v>
+      </x:c>
+      <x:c r="B19" s="16" t="str">
+        <x:v>[BB]</x:v>
+      </x:c>
+      <x:c r="C19" s="16" t="str">
+        <x:v>11/10/2026</x:v>
+      </x:c>
+      <x:c r="D19" s="17" t="d">
+        <x:v>2026-10-13T09:02:31.820Z</x:v>
+      </x:c>
+      <x:c r="E19" s="17" t="d">
+        <x:v>2026-10-13T09:09:38.073Z</x:v>
+      </x:c>
+      <x:c r="F19" s="18" t="n">
+        <x:v>0.00493349537037037</x:v>
+      </x:c>
+      <x:c r="G19" s="16" t="str">
+        <x:v>สำเร็จ</x:v>
+      </x:c>
+      <x:c r="H19" s="16" t="str">
+        <x:v>ประมวลผลและกด Finish แล้ว</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="19" t="str">
+        <x:v>20261013-090231</x:v>
+      </x:c>
+      <x:c r="B20" s="19" t="str">
+        <x:v>[BK]</x:v>
+      </x:c>
+      <x:c r="C20" s="19" t="str">
+        <x:v>11/10/2026</x:v>
+      </x:c>
+      <x:c r="D20" s="20" t="d">
+        <x:v>2026-10-13T09:09:45.765Z</x:v>
+      </x:c>
+      <x:c r="E20" s="20" t="d">
+        <x:v>2026-10-13T09:22:03.629Z</x:v>
+      </x:c>
+      <x:c r="F20" s="21" t="n">
+        <x:v>0.008540092592592592</x:v>
+      </x:c>
+      <x:c r="G20" s="19" t="str">
+        <x:v>สำเร็จ</x:v>
+      </x:c>
+      <x:c r="H20" s="19" t="str">
+        <x:v>ประมวลผลและกด Finish แล้ว</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="16" t="str">
+        <x:v>20261013-090231</x:v>
+      </x:c>
+      <x:c r="B21" s="16" t="str">
+        <x:v>[NTS]</x:v>
+      </x:c>
+      <x:c r="C21" s="16" t="str">
+        <x:v>11/10/2026</x:v>
+      </x:c>
+      <x:c r="D21" s="17" t="d">
+        <x:v>2026-10-13T09:22:11.344Z</x:v>
+      </x:c>
+      <x:c r="E21" s="17" t="d">
+        <x:v>2026-10-13T09:23:15.334Z</x:v>
+      </x:c>
+      <x:c r="F21" s="18" t="n">
+        <x:v>0.0007406018518518519</x:v>
+      </x:c>
+      <x:c r="G21" s="16" t="str">
+        <x:v>สำเร็จ</x:v>
+      </x:c>
+      <x:c r="H21" s="16" t="str">
+        <x:v>ประมวลผลและกด Finish แล้ว</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="19" t="str">
+        <x:v>20261013-090231</x:v>
+      </x:c>
+      <x:c r="B22" s="19" t="str">
+        <x:v>[PK]</x:v>
+      </x:c>
+      <x:c r="C22" s="19" t="str">
+        <x:v>11/10/2026</x:v>
+      </x:c>
+      <x:c r="D22" s="20" t="d">
+        <x:v>2026-10-13T09:23:22.768Z</x:v>
+      </x:c>
+      <x:c r="E22" s="20" t="d">
+        <x:v>2026-10-13T09:25:39.913Z</x:v>
+      </x:c>
+      <x:c r="F22" s="21" t="n">
+        <x:v>0.001587326388888889</x:v>
+      </x:c>
+      <x:c r="G22" s="19" t="str">
+        <x:v>สำเร็จ</x:v>
+      </x:c>
+      <x:c r="H22" s="19" t="str">
+        <x:v>ประมวลผลและกด Finish แล้ว</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="16" t="str">
+        <x:v>20261013-090231</x:v>
+      </x:c>
+      <x:c r="B23" s="16" t="str">
+        <x:v>[SM]</x:v>
+      </x:c>
+      <x:c r="C23" s="16" t="str">
+        <x:v>11/10/2026</x:v>
+      </x:c>
+      <x:c r="D23" s="17" t="d">
+        <x:v>2026-10-13T09:25:47.687Z</x:v>
+      </x:c>
+      <x:c r="E23" s="17" t="d">
+        <x:v>2026-10-13T09:27:56.494Z</x:v>
+      </x:c>
+      <x:c r="F23" s="18" t="n">
+        <x:v>0.0014908217592592592</x:v>
+      </x:c>
+      <x:c r="G23" s="16" t="str">
+        <x:v>สำเร็จ</x:v>
+      </x:c>
+      <x:c r="H23" s="16" t="str">
+        <x:v>ประมวลผลและกด Finish แล้ว</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="28" t="str">
+        <x:v>20261013-090231</x:v>
+      </x:c>
+      <x:c r="B24" s="28" t="str">
+        <x:v>สรุปรอบ</x:v>
+      </x:c>
+      <x:c r="C24" s="28" t="str">
+        <x:v>11/10/2026</x:v>
+      </x:c>
+      <x:c r="D24" s="29" t="d">
+        <x:v>2026-10-13T09:02:31.820Z</x:v>
+      </x:c>
+      <x:c r="E24" s="29" t="d">
+        <x:v>2026-10-13T09:27:56.494Z</x:v>
+      </x:c>
+      <x:c r="F24" s="30" t="n">
+        <x:v>0.017646701388888887</x:v>
+      </x:c>
+      <x:c r="G24" s="28" t="str">
+        <x:v>สำเร็จครบ 5 สาขา</x:v>
+      </x:c>
+      <x:c r="H24" s="28" t="str">
+        <x:v>รวมตั้งแต่เริ่ม [BB] ถึง Finish [SM]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="16" t="str">
+        <x:v>20261013-101514</x:v>
+      </x:c>
+      <x:c r="B25" s="16" t="str">
+        <x:v>[BB]</x:v>
+      </x:c>
+      <x:c r="C25" s="16" t="str">
+        <x:v>10/10/2026 - 11/10/2026</x:v>
+      </x:c>
+      <x:c r="D25" s="17" t="d">
+        <x:v>2026-10-13T10:15:20.256Z</x:v>
+      </x:c>
+      <x:c r="E25" s="17" t="d">
+        <x:v>2026-10-13T10:23:02.873Z</x:v>
+      </x:c>
+      <x:c r="F25" s="18" t="n">
+        <x:v>0.0053543634259259265</x:v>
+      </x:c>
+      <x:c r="G25" s="16" t="str">
+        <x:v>สำเร็จ</x:v>
+      </x:c>
+      <x:c r="H25" s="16" t="str">
+        <x:v>ประมวลผลและกด Finish แล้ว</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="19" t="str">
+        <x:v>20261013-101514</x:v>
+      </x:c>
+      <x:c r="B26" s="19" t="str">
+        <x:v>[BK]</x:v>
+      </x:c>
+      <x:c r="C26" s="19" t="str">
+        <x:v>10/10/2026 - 11/10/2026</x:v>
+      </x:c>
+      <x:c r="D26" s="20" t="d">
+        <x:v>2026-10-13T10:23:11.857Z</x:v>
+      </x:c>
+      <x:c r="E26" s="20" t="d">
+        <x:v>2026-10-13T10:36:24.196Z</x:v>
+      </x:c>
+      <x:c r="F26" s="21" t="n">
+        <x:v>0.00917059027777778</x:v>
+      </x:c>
+      <x:c r="G26" s="19" t="str">
+        <x:v>สำเร็จ</x:v>
+      </x:c>
+      <x:c r="H26" s="19" t="str">
+        <x:v>ประมวลผลและกด Finish แล้ว</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="16" t="str">
+        <x:v>20261013-101514</x:v>
+      </x:c>
+      <x:c r="B27" s="16" t="str">
+        <x:v>[NTS]</x:v>
+      </x:c>
+      <x:c r="C27" s="16" t="str">
+        <x:v>10/10/2026 - 11/10/2026</x:v>
+      </x:c>
+      <x:c r="D27" s="17" t="d">
+        <x:v>2026-10-13T10:36:32.936Z</x:v>
+      </x:c>
+      <x:c r="E27" s="17" t="d">
+        <x:v>2026-10-13T10:37:43.349Z</x:v>
+      </x:c>
+      <x:c r="F27" s="18" t="n">
+        <x:v>0.0008149652777777777</x:v>
+      </x:c>
+      <x:c r="G27" s="16" t="str">
+        <x:v>สำเร็จ</x:v>
+      </x:c>
+      <x:c r="H27" s="16" t="str">
+        <x:v>ประมวลผลและกด Finish แล้ว</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="19" t="str">
+        <x:v>20261013-101514</x:v>
+      </x:c>
+      <x:c r="B28" s="19" t="str">
+        <x:v>[PK]</x:v>
+      </x:c>
+      <x:c r="C28" s="19" t="str">
+        <x:v>10/10/2026 - 11/10/2026</x:v>
+      </x:c>
+      <x:c r="D28" s="20" t="d">
+        <x:v>2026-10-13T10:37:51.837Z</x:v>
+      </x:c>
+      <x:c r="E28" s="20" t="d">
+        <x:v>2026-10-13T10:40:22.366Z</x:v>
+      </x:c>
+      <x:c r="F28" s="21" t="n">
+        <x:v>0.001742222222222222</x:v>
+      </x:c>
+      <x:c r="G28" s="19" t="str">
+        <x:v>สำเร็จ</x:v>
+      </x:c>
+      <x:c r="H28" s="19" t="str">
+        <x:v>ประมวลผลและกด Finish แล้ว</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="16" t="str">
+        <x:v>20261013-101514</x:v>
+      </x:c>
+      <x:c r="B29" s="16" t="str">
+        <x:v>[SM]</x:v>
+      </x:c>
+      <x:c r="C29" s="16" t="str">
+        <x:v>10/10/2026 - 11/10/2026</x:v>
+      </x:c>
+      <x:c r="D29" s="17" t="d">
+        <x:v>2026-10-13T10:40:30.669Z</x:v>
+      </x:c>
+      <x:c r="E29" s="17" t="d">
+        <x:v>2026-10-13T10:42:50.040Z</x:v>
+      </x:c>
+      <x:c r="F29" s="18" t="n">
+        <x:v>0.001613090277777778</x:v>
+      </x:c>
+      <x:c r="G29" s="16" t="str">
+        <x:v>สำเร็จ</x:v>
+      </x:c>
+      <x:c r="H29" s="16" t="str">
+        <x:v>ประมวลผลและกด Finish แล้ว</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="28" t="str">
+        <x:v>20261013-101514</x:v>
+      </x:c>
+      <x:c r="B30" s="28" t="str">
+        <x:v>สรุปรอบ</x:v>
+      </x:c>
+      <x:c r="C30" s="28" t="str">
+        <x:v>10/10/2026 - 11/10/2026</x:v>
+      </x:c>
+      <x:c r="D30" s="29" t="d">
+        <x:v>2026-10-13T10:15:20.256Z</x:v>
+      </x:c>
+      <x:c r="E30" s="29" t="d">
+        <x:v>2026-10-13T10:42:50.040Z</x:v>
+      </x:c>
+      <x:c r="F30" s="30" t="n">
+        <x:v>0.019094722222222225</x:v>
+      </x:c>
+      <x:c r="G30" s="28" t="str">
+        <x:v>สำเร็จครบ 5 สาขา</x:v>
+      </x:c>
+      <x:c r="H30" s="28" t="str">
         <x:v>รวมตั้งแต่เริ่ม [BB] ถึง Finish [SM]</x:v>
       </x:c>
     </x:row>
@@ -680,7 +1184,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="G5:G10">
+  <x:conditionalFormatting sqref="G5:G30">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="สำเร็จ"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="ผิดพลาด"/>
   </x:conditionalFormatting>

</xml_diff>

<commit_message>
Update HRMI processing times
</commit_message>
<xml_diff>
--- a/HRMI-processing-times.xlsx
+++ b/HRMI-processing-times.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="เวลาประมวลผล" sheetId="1" r:id="Re4c7d3d2c0d44dc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="เวลาประมวลผล" sheetId="1" r:id="Ree94ad7be2204d7a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1180,11 +1180,37 @@
         <x:v>รวมตั้งแต่เริ่ม [BB] ถึง Finish [SM]</x:v>
       </x:c>
     </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="16" t="str">
+        <x:v>20261014-080324</x:v>
+      </x:c>
+      <x:c r="B31" s="16" t="str">
+        <x:v>[BB]</x:v>
+      </x:c>
+      <x:c r="C31" s="16" t="str">
+        <x:v>12/10/2026</x:v>
+      </x:c>
+      <x:c r="D31" s="17" t="d">
+        <x:v>2026-10-14T08:03:30.827Z</x:v>
+      </x:c>
+      <x:c r="E31" s="17" t="d">
+        <x:v>2026-10-14T08:05:01.401Z</x:v>
+      </x:c>
+      <x:c r="F31" s="18" t="n">
+        <x:v>0.0010483101851851851</x:v>
+      </x:c>
+      <x:c r="G31" s="16" t="str">
+        <x:v>ผิดพลาด</x:v>
+      </x:c>
+      <x:c r="H31" s="16" t="str">
+        <x:v>ปรับเทียบไม่สำเร็จ: ไม่พบการคลิกหรือหน้า Time Attendance Flow</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="G5:G30">
+  <x:conditionalFormatting sqref="G5:G31">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="สำเร็จ"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="ผิดพลาด"/>
   </x:conditionalFormatting>

</xml_diff>